<commit_message>
Update v18.50: All Excel files updated with Province, popup order fixed (Locality, Municipality, Province), and code cleanup
</commit_message>
<xml_diff>
--- a/Pipistrelli 2022.xlsx
+++ b/Pipistrelli 2022.xlsx
@@ -629,7 +629,11 @@
           <t>Sarcedo</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
       <c r="H4" t="n">
         <v>45.7104304</v>
       </c>
@@ -801,7 +805,11 @@
           <t>Malo</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>VI</t>
+        </is>
+      </c>
       <c r="H7" t="n">
         <v>45.6577546</v>
       </c>

</xml_diff>